<commit_message>
End of session — Claude Code setup restructured: MCP fixed at user scope, CLAUDE.md hierarchy deduplicated, agents rewritten + research family created, QA checklists added, web search made backend-agnostic
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hseea/Docs to add to the Knowledge store.xlsx
+++ b/hseea/Docs to add to the Knowledge store.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\terminai\hseea\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2FB7C1AA-BDF6-42F8-9C03-BA464804FD96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D577998-33AF-4CC8-AB23-8F8A3FB1F92E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-25710" yWindow="-60" windowWidth="21600" windowHeight="11295" xr2:uid="{230B636A-538C-4359-83A5-B4D6DC444691}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="30">
   <si>
     <t>HSE</t>
   </si>
@@ -123,6 +123,12 @@
   </si>
   <si>
     <t>github-markdown.pdf</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Done</t>
   </si>
 </sst>
 </file>
@@ -586,32 +592,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AB72B40-3049-4DA3-B258-31DE7B1F86F3}">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="75.5703125" customWidth="1"/>
-    <col min="2" max="3" width="114.5703125" customWidth="1"/>
+    <col min="2" max="2" width="29.5703125" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4"/>
       <c r="B1" s="5"/>
     </row>
-    <row r="2" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7"/>
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" s="8" customFormat="1" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" s="8" customFormat="1" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -619,23 +629,29 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>26</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>8</v>
       </c>
@@ -643,7 +659,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:2" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>10</v>
       </c>
@@ -651,7 +667,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:2" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>12</v>
       </c>
@@ -659,7 +675,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:2" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>14</v>
       </c>
@@ -667,7 +683,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:2" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>15</v>
       </c>
@@ -675,7 +691,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:2" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
         <v>17</v>
       </c>
@@ -683,7 +699,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:2" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
         <v>19</v>
       </c>
@@ -691,7 +707,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:2" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
         <v>20</v>
       </c>
@@ -699,7 +715,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:2" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
         <v>21</v>
       </c>
@@ -707,7 +723,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:2" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" s="8" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
         <v>22</v>
       </c>

</xml_diff>